<commit_message>
chore(release): verify and finish all training material platform features
</commit_message>
<xml_diff>
--- a/教育訓練教材/backend/chat_logs.xlsx
+++ b/教育訓練教材/backend/chat_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,32 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-06 15:17:48</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.一階調撥.md</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>是否能幫我美化圖片</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>學員您好！
+很抱歉，我是企業內訓的 AI 助教，目前主要協助解答內部訓練教材相關的問題（例如：ERP 倉儲單據作業流程、三合一對刷系統操作、迎新與公司規範等）。
+由於**「圖片美化」**不在本次的教材與系統服務範圍內，我無法直接幫您修圖或美化圖片。建議您可以使用專門的影像處理軟體或圖片編輯工具來進行處理。
+如果您在閱讀教材或操作內部系統時有任何疑問，隨時歡迎向我提問，我很樂意為您解答！
+*(Powered by gemini-3.8-flash / Key: AQ.A...wlGw)*</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>